<commit_message>
Added More Technical Questions per SubjectMatter
</commit_message>
<xml_diff>
--- a/technical_assessment_by_job/questions/git_questions.xlsx
+++ b/technical_assessment_by_job/questions/git_questions.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ws_openai_ws\technical_assessment_by_job\questions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ws_openai\codex_projects\technical_assessment_by_job\questions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6CD37373-67E3-4ADB-B8A9-786EBAF59296}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{186133B6-0F4E-4E66-BD8D-8BED2E73F901}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{A23630A7-5661-4D23-87E6-A5D22EEBE10B}"/>
   </bookViews>
@@ -35,10 +35,452 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="143">
+  <si>
+    <t>Question</t>
+  </si>
+  <si>
+    <t>Answer</t>
+  </si>
+  <si>
+    <t>What is Git?</t>
+  </si>
+  <si>
+    <t>Git is an open-source distributed version control system (VCS) used to track changes in source code during software development. It allows multiple developers to work together on the same project.</t>
+  </si>
+  <si>
+    <t>What is a Version Control System (VCS)?</t>
+  </si>
+  <si>
+    <t>A VCS is software that tracks and manages changes to a file system. It records who made changes, what changes were made, and allows you to revert to previous versions.</t>
+  </si>
+  <si>
+    <t>Difference between Git and SVN?</t>
+  </si>
+  <si>
+    <t>Git is distributed (every developer has a local copy of the entire history), while SVN is centralized (history is only on a central server). Git is generally faster and handles branching better.</t>
+  </si>
+  <si>
+    <t>What is a Repository in Git?</t>
+  </si>
+  <si>
+    <t>A repository (repo) is a directory or storage space where Git tracks all project files and their history. It contains a .git folder with metadata.</t>
+  </si>
+  <si>
+    <t>What is 'bare' repository in Git?</t>
+  </si>
+  <si>
+    <t>A bare repository is a repository that doesn't have a working directory. It only contains the version control information (.git folder contents). It's typically used as a central server for sharing.</t>
+  </si>
+  <si>
+    <t>What is 'index' or 'staging area'?</t>
+  </si>
+  <si>
+    <t>The staging area is an intermediate area where files are formatted and prepared before they are committed to the repository.</t>
+  </si>
+  <si>
+    <t>What is 'commit' in Git?</t>
+  </si>
+  <si>
+    <t>A commit is a snapshot of your changes at a specific point in time. Each commit has a unique SHA-1 hash ID.</t>
+  </si>
+  <si>
+    <t>How do you initialize a new Git repository?</t>
+  </si>
+  <si>
+    <t>By using the command: git init</t>
+  </si>
+  <si>
+    <t>What is the use of 'git config'?</t>
+  </si>
+  <si>
+    <t>It is used to set configuration options for your Git installation, such as user name, email, and preferred editor.</t>
+  </si>
+  <si>
+    <t>How to check the status of files in Git?</t>
+  </si>
+  <si>
+    <t>Use the command: git status</t>
+  </si>
+  <si>
+    <t>What is 'git add'?</t>
+  </si>
+  <si>
+    <t>It adds file changes in your working directory to your index (staging area).</t>
+  </si>
+  <si>
+    <t>What is 'git commit -m'?</t>
+  </si>
+  <si>
+    <t>It creates a commit with a message describing the changes made.</t>
+  </si>
+  <si>
+    <t>What is 'git log'?</t>
+  </si>
+  <si>
+    <t>It displays the history of commits for the current branch.</t>
+  </si>
+  <si>
+    <t>What is 'git diff'?</t>
+  </si>
+  <si>
+    <t>It shows the differences between the working directory, staging area, and the last commit.</t>
+  </si>
+  <si>
+    <t>What is a Branch in Git?</t>
+  </si>
+  <si>
+    <t>A branch is a lightweight movable pointer to a commit. It allows you to develop features or fix bugs in isolation from the main codebase (master/main).</t>
+  </si>
+  <si>
+    <t>How do you create a new branch?</t>
+  </si>
+  <si>
+    <t>git branch &lt;branch_name&gt;</t>
+  </si>
+  <si>
+    <t>How do you switch to a branch?</t>
+  </si>
+  <si>
+    <t>git checkout &lt;branch_name&gt; (or git switch &lt;branch_name&gt; in newer versions).</t>
+  </si>
+  <si>
+    <t>What is 'git merge'?</t>
+  </si>
+  <si>
+    <t>It combines the changes from one branch into another (e.g., merging a feature branch into main).</t>
+  </si>
+  <si>
+    <t>What is a Merge Conflict?</t>
+  </si>
+  <si>
+    <t>A conflict occurs when two branches have different changes to the same line of a file, and Git cannot automatically determine which version to keep.</t>
+  </si>
+  <si>
+    <t>How do you delete a branch?</t>
+  </si>
+  <si>
+    <t>git branch -d &lt;branch_name&gt;</t>
+  </si>
+  <si>
+    <t>What is 'git clone'?</t>
+  </si>
+  <si>
+    <t>It creates a local copy of an existing remote repository.</t>
+  </si>
+  <si>
+    <t>What is 'git push'?</t>
+  </si>
+  <si>
+    <t>It uploads local repository commits to a remote repository.</t>
+  </si>
+  <si>
+    <t>What is 'git pull'?</t>
+  </si>
+  <si>
+    <t>It fetches changes from a remote repository and immediately merges them into your local branch (fetch + merge).</t>
+  </si>
+  <si>
+    <t>What is 'git fetch'?</t>
+  </si>
+  <si>
+    <t>It downloads changes from the remote repository but does not merge them into your local work.</t>
+  </si>
+  <si>
+    <t>What is 'git remote'?</t>
+  </si>
+  <si>
+    <t>It is used to manage connections to remote repositories.</t>
+  </si>
+  <si>
+    <t>What is Git Stash?</t>
+  </si>
+  <si>
+    <t>Stashing takes your uncommitted changes (both staged and unstaged) and saves them for later use, cleaning up your working directory.</t>
+  </si>
+  <si>
+    <t>How to bring back stashed changes?</t>
+  </si>
+  <si>
+    <t>git stash pop (applies and removes from stash) or git stash apply (applies but keeps in stash).</t>
+  </si>
+  <si>
+    <t>What is 'git rebase'?</t>
+  </si>
+  <si>
+    <t>Rebasing is the process of moving or combining a sequence of commits to a new base commit. It creates a linear history.</t>
+  </si>
+  <si>
+    <t>Rebase vs Merge?</t>
+  </si>
+  <si>
+    <t>Merge keeps the history of both branches and creates a merge commit. Rebase rewrites history to create a clean, linear path.</t>
+  </si>
+  <si>
+    <t>What is 'git cherry-pick'?</t>
+  </si>
+  <si>
+    <t>It allows you to pick a specific commit from one branch and apply it to another.</t>
+  </si>
+  <si>
+    <t>What is 'git revert'?</t>
+  </si>
+  <si>
+    <t>It creates a new commit that undoes the changes of a previous commit without deleting the history.</t>
+  </si>
+  <si>
+    <t>What is 'git reset'?</t>
+  </si>
+  <si>
+    <t>It moves the current branch head to a specific commit. It can be --soft, --mixed, or --hard.</t>
+  </si>
+  <si>
+    <t>Difference between 'git reset' and 'git revert'?</t>
+  </si>
+  <si>
+    <t>Reset moves the pointer backward (potentially losing work), while revert adds a new commit to undo changes (safe for shared branches).</t>
+  </si>
+  <si>
+    <t>What is 'git tag'?</t>
+  </si>
+  <si>
+    <t>Tags are used to mark specific points in history as important, usually for version releases (e.g., v1.0).</t>
+  </si>
+  <si>
+    <t>What are Git Hooks?</t>
+  </si>
+  <si>
+    <t>Scripts that Git executes before or after events like commit, push, and receive (e.g., pre-commit hooks for linting).</t>
+  </si>
+  <si>
+    <t>What is .gitignore?</t>
+  </si>
+  <si>
+    <t>A file that tells Git which files or directories to ignore and not track (e.g., node_modules, log files).</t>
+  </si>
+  <si>
+    <t>What is 'git reflog'?</t>
+  </si>
+  <si>
+    <t>It records every time the HEAD of a branch is updated. It's useful for recovering lost commits or deleted branches.</t>
+  </si>
+  <si>
+    <t>What is 'git am'?</t>
+  </si>
+  <si>
+    <t>It is used to apply a series of patches from a mailbox.</t>
+  </si>
+  <si>
+    <t>How to rename a branch?</t>
+  </si>
+  <si>
+    <t>git branch -m &lt;old_name&gt; &lt;new_name&gt;</t>
+  </si>
+  <si>
+    <t>How to change the last commit message?</t>
+  </si>
+  <si>
+    <t>git commit --amend -m 'New message'</t>
+  </si>
+  <si>
+    <t>What is the 'HEAD' in Git?</t>
+  </si>
+  <si>
+    <t>HEAD is a reference to the last commit in the currently checked-out branch.</t>
+  </si>
+  <si>
+    <t>What is 'detached HEAD'?</t>
+  </si>
+  <si>
+    <t>It happens when you check out a specific commit or tag instead of a branch. Changes made here won't belong to any branch.</t>
+  </si>
+  <si>
+    <t>What is a Git Submodule?</t>
+  </si>
+  <si>
+    <t>It allows you to keep another Git repository as a subdirectory of your own repository, often used for shared libraries.</t>
+  </si>
+  <si>
+    <t>What is the Git workflow 'Gitflow'?</t>
+  </si>
+  <si>
+    <t>A branching model that uses 'develop', 'main', 'feature', 'release', and 'hotfix' branches to manage complex releases.</t>
+  </si>
+  <si>
+    <t>What is 'git bisect'?</t>
+  </si>
+  <si>
+    <t>A binary search tool used to find the specific commit that introduced a bug.</t>
+  </si>
+  <si>
+    <t>How to squashing commits?</t>
+  </si>
+  <si>
+    <t>Using interactive rebase: git rebase -i HEAD~n, then changing 'pick' to 'squash' for the desired commits.</t>
+  </si>
+  <si>
+    <t>What is 'git archive'?</t>
+  </si>
+  <si>
+    <t>Creates an archive (zip/tar) of the files in a specific tree or commit, excluding Git metadata.</t>
+  </si>
+  <si>
+    <t>What is 'git show'?</t>
+  </si>
+  <si>
+    <t>Shows various types of objects (commits, tags, etc.) and their specific changes.</t>
+  </si>
+  <si>
+    <t>What is 'git blame'?</t>
+  </si>
+  <si>
+    <t>It shows who last modified each line of a file and in which commit.</t>
+  </si>
+  <si>
+    <t>How to recover a deleted branch?</t>
+  </si>
+  <si>
+    <t>Find the commit hash in 'git reflog' and run 'git checkout -b &lt;branch_name&gt; &lt;hash&gt;'.</t>
+  </si>
+  <si>
+    <t>What is the difference between 'git pull' and 'git fetch'?</t>
+  </si>
+  <si>
+    <t>Fetch only downloads data; pull downloads and automatically attempts to merge it into your current branch.</t>
+  </si>
+  <si>
+    <t>What is a 'conflict resolution strategy'?</t>
+  </si>
+  <si>
+    <t>Approaches like 'ours' (keep current branch version) or 'theirs' (keep incoming branch version) used during merges.</t>
+  </si>
+  <si>
+    <t>What is Git LFS?</t>
+  </si>
+  <si>
+    <t>Git Large File Storage; it replaces large files with text pointers inside Git, storing the file contents on a remote server.</t>
+  </si>
+  <si>
+    <t>What is the '.git' directory?</t>
+  </si>
+  <si>
+    <t>The hidden directory where Git stores all its data, configuration, and compressed objects.</t>
+  </si>
+  <si>
+    <t>How to push a local branch to a remote for the first time?</t>
+  </si>
+  <si>
+    <t>git push -u origin &lt;branch_name&gt;</t>
+  </si>
+  <si>
+    <t>What is 'git help'?</t>
+  </si>
+  <si>
+    <t>Displays manual pages for Git commands.</t>
+  </si>
+  <si>
+    <t>What is a 'fast-forward' merge?</t>
+  </si>
+  <si>
+    <t>A merge where the target branch has not diverged; Git simply moves the pointer forward to the new commit.</t>
+  </si>
+  <si>
+    <t>What is 'git clean'?</t>
+  </si>
+  <si>
+    <t>Removes untracked files from the working directory.</t>
+  </si>
+  <si>
+    <t>How to stage only a portion of a file?</t>
+  </si>
+  <si>
+    <t>git add -p (patch mode).</t>
+  </si>
+  <si>
+    <t>What is the 'three-tree architecture' of Git?</t>
+  </si>
+  <si>
+    <t>Working Directory, Staging Area (Index), and Repository (HEAD).</t>
+  </si>
+  <si>
+    <t>Explain SHA-1 in Git.</t>
+  </si>
+  <si>
+    <t>Git uses SHA-1 hashing to identify every commit, tree, and file uniquely based on its content.</t>
+  </si>
+  <si>
+    <t>What is 'git fsck'?</t>
+  </si>
+  <si>
+    <t>File System Check; it verifies the connectivity and validity of objects in the database.</t>
+  </si>
+  <si>
+    <t>What is 'git gc'?</t>
+  </si>
+  <si>
+    <t>Garbage Collector; it cleans up unnecessary files and optimizes the local repository.</t>
+  </si>
+  <si>
+    <t>How to check which branches have been merged?</t>
+  </si>
+  <si>
+    <t>git branch --merged</t>
+  </si>
+  <si>
+    <t>How to view the commit history as a graph?</t>
+  </si>
+  <si>
+    <t>git log --graph --oneline --all</t>
+  </si>
+  <si>
+    <t>What is 'git bundle'?</t>
+  </si>
+  <si>
+    <t>It packages objects and references into a single file to share history without a network connection.</t>
+  </si>
+  <si>
+    <t>Difference between SSH and HTTPS for remote?</t>
+  </si>
+  <si>
+    <t>HTTPS is easier to set up behind firewalls; SSH is more secure and doesn't require repeated password entry with keys.</t>
+  </si>
+  <si>
+    <t>What is a 'fork'?</t>
+  </si>
+  <si>
+    <t>A copy of a repository hosted on a service like GitHub, allowing you to make changes without affecting the original project.</t>
+  </si>
+  <si>
+    <t>What is a Pull Request (PR)?</t>
+  </si>
+  <si>
+    <t>A method of submitting contributions to an open-source project or within a team, where changes are reviewed before merging.</t>
+  </si>
+  <si>
+    <t>Can you explain 'git worktree'?</t>
+  </si>
+  <si>
+    <t>It allows you to have multiple working trees attached to the same repository, so you can check out multiple branches at once in different folders.</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -54,7 +496,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -62,12 +504,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -402,9 +869,794 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4113CA9F-0F03-4B84-B554-4651E8B0FDDD}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="8.7265625" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="4">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="4">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="4">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="4">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="4">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="4">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="4">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="4">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="4">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="4">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="4">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="4">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="4">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="4">
+        <v>15</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" s="4">
+        <v>16</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" s="4">
+        <v>17</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" s="4">
+        <v>18</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" s="4">
+        <v>19</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" s="4">
+        <v>20</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" s="4">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" s="4">
+        <v>22</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" s="4">
+        <v>23</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" s="4">
+        <v>24</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A26" s="4">
+        <v>25</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27" s="4">
+        <v>26</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A28" s="4">
+        <v>27</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A29" s="4">
+        <v>28</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A30" s="4">
+        <v>29</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31" s="4">
+        <v>30</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A32" s="4">
+        <v>31</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" s="4">
+        <v>32</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34" s="4">
+        <v>33</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A35" s="4">
+        <v>34</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A36" s="4">
+        <v>35</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A37" s="4">
+        <v>36</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38" s="4">
+        <v>37</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A39" s="4">
+        <v>38</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A40" s="4">
+        <v>39</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A41" s="4">
+        <v>40</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A42" s="4">
+        <v>41</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A43" s="4">
+        <v>42</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A44" s="4">
+        <v>43</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A45" s="4">
+        <v>44</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A46" s="4">
+        <v>45</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A47" s="4">
+        <v>46</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A48" s="4">
+        <v>47</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A49" s="4">
+        <v>48</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A50" s="4">
+        <v>49</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A51" s="4">
+        <v>50</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A52" s="4">
+        <v>51</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A53" s="4">
+        <v>52</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A54" s="4">
+        <v>53</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A55" s="4">
+        <v>54</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A56" s="4">
+        <v>55</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A57" s="4">
+        <v>56</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A58" s="4">
+        <v>57</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A59" s="4">
+        <v>58</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A60" s="4">
+        <v>59</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A61" s="4">
+        <v>60</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A62" s="4">
+        <v>61</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A63" s="4">
+        <v>62</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A64" s="4">
+        <v>63</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A65" s="4">
+        <v>64</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A66" s="4">
+        <v>65</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A67" s="4">
+        <v>66</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A68" s="4">
+        <v>67</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A69" s="4">
+        <v>68</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A70" s="4">
+        <v>69</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A71" s="4">
+        <v>70</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>